<commit_message>
v4 logs 2026-07-22 18:42 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -536,17 +536,68 @@
           <t>Sent 1 GEMS - None</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>ARB-USD:6</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>00:12:16 IST</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sent 1 GEMS - None</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>ARB-USD:6</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -610,10 +661,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -622,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 18:46 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -587,17 +587,68 @@
           <t>Sent 1 GEMS - None</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>ARB-USD:6</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>00:16:22 IST</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sent 1 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>ARB-USD:6</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -661,10 +712,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -673,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 19:03 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -638,17 +638,68 @@
           <t>Sent 1 GEMS - 200</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ARB-USD:6</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>00:33:50 IST</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Sent 1 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>ARB-USD:6</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -712,10 +763,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -724,7 +775,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 19:22 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,17 +689,68 @@
           <t>Sent 1 GEMS - 200</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>ARB-USD:6</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>00:52:13 IST</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Sent 12 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>ARB-USD:6</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -763,10 +814,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -775,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -792,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -915,6 +966,198 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>00:52:19 IST</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AAVE-USD</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>97.87000274658205</v>
+      </c>
+      <c r="F3" t="n">
+        <v>510</v>
+      </c>
+      <c r="G3" t="n">
+        <v>95.91</v>
+      </c>
+      <c r="H3" t="n">
+        <v>101.78</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Trend Pullback, RSI 63 Score:3 RVOL:1.4x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>00:52:19 IST</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ADA-USD</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1745000034570694</v>
+      </c>
+      <c r="F4" t="n">
+        <v>222222</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Trend Pullback, RSI 60 Score:3 RVOL:0.8x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>00:52:19 IST</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HBAR-USD</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0717300027608871</v>
+      </c>
+      <c r="F5" t="n">
+        <v>578033</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>00:52:19 IST</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BTC-USD</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>65805.859375</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>64489.74</v>
+      </c>
+      <c r="H6" t="n">
+        <v>68438.09</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>RSI 66, EMA Bull Score:2 RVOL:1.1x</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 19:31 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -740,17 +740,68 @@
           <t>Sent 12 GEMS - 200</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01:01:20 IST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>13</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Sent 13 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -814,10 +865,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -826,7 +877,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -843,7 +894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1095,18 +1146,28 @@
       <c r="H5" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>01:01:23 IST</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-2.41</v>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x</t>
+          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x | Target Hit</t>
         </is>
       </c>
     </row>
@@ -1158,6 +1219,54 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01:01:23 IST</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HBAR-USD</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.07169</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.070256</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.074558</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 19:39 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -791,17 +791,68 @@
           <t>Sent 13 GEMS - 200</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01:09:40 IST</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>13</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>13</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sent 13 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -865,10 +916,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -877,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 19:56 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -842,17 +842,68 @@
           <t>Sent 13 GEMS - 200</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>01:25:56 IST</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>13</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Sent 13 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -916,10 +967,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -928,7 +979,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -945,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1028,7 +1079,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00:01:28 IST</t>
+          <t>01:26:00 IST</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1042,16 +1093,16 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.0007570616435258999</v>
+        <v>0.00075706</v>
       </c>
       <c r="F2" t="n">
-        <v>1320896</v>
+        <v>5000</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.00074192</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>0.00078734</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -1064,7 +1115,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>RVOL 20.0x, 20D Break 0&gt;0 Score:6 RVOL:20.0x</t>
+          <t>RVOL 15.0x, 20D Breakout Score:7 RVOL:15.0x</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>00:52:19 IST</t>
+          <t>01:26:00 IST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1090,16 +1141,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>97.87000274658205</v>
+        <v>97.84</v>
       </c>
       <c r="F3" t="n">
-        <v>510</v>
+        <v>204</v>
       </c>
       <c r="G3" t="n">
-        <v>95.91</v>
+        <v>95.88</v>
       </c>
       <c r="H3" t="n">
-        <v>101.78</v>
+        <v>101.75</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -1124,7 +1175,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>00:52:19 IST</t>
+          <t>01:26:00 IST</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1138,16 +1189,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.1745000034570694</v>
+        <v>0.1744</v>
       </c>
       <c r="F4" t="n">
-        <v>222222</v>
+        <v>10000</v>
       </c>
       <c r="G4" t="n">
-        <v>0.17</v>
+        <v>0.1709</v>
       </c>
       <c r="H4" t="n">
-        <v>0.18</v>
+        <v>0.1814</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -1172,7 +1223,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>00:52:19 IST</t>
+          <t>01:26:00 IST</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1186,39 +1237,29 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.0717300027608871</v>
+        <v>0.07167</v>
       </c>
       <c r="F5" t="n">
-        <v>578033</v>
+        <v>5000</v>
       </c>
       <c r="G5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.07023699999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>01:01:23 IST</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="L5" t="n">
-        <v>-2.41</v>
-      </c>
+        <v>0.07453700000000001</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x | Target Hit</t>
+          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1271,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>00:52:19 IST</t>
+          <t>01:26:00 IST</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1244,16 +1285,16 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>65805.859375</v>
+        <v>65880.89999999999</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>64489.74</v>
+        <v>64563.28</v>
       </c>
       <c r="H6" t="n">
-        <v>68438.09</v>
+        <v>68516.14</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -1270,54 +1311,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>01:01:23 IST</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CRYPTO</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>HBAR-USD</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.07169</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.070256</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.074558</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>VWAP Reclaim, RSI 58 Score:2 RVOL:1.6x</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 21:05 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -893,17 +893,68 @@
           <t>Sent 13 GEMS - 200</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>02:35:44 IST</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>13</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>13</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Sent 13 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -967,10 +1018,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C2" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -979,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-22 23:01 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,17 +944,68 @@
           <t>Sent 13 GEMS - 200</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:31:52 IST</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>13</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>13</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sent 13 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -1018,10 +1069,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="C2" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1030,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v4 logs 2026-07-23 02:37 UTC
</commit_message>
<xml_diff>
--- a/logs/trade_log.xlsx
+++ b/logs/trade_log.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -995,17 +995,68 @@
           <t>Sent 13 GEMS - 200</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:06:59 IST</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CRYPTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>12</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Sent 12 GEMS - 200</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>ARB-USD:7 | AAVE-USD:3 | ADA-USD:3 | HBAR-USD:2 | BTC-USD:2</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -1069,10 +1120,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C2" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1081,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>

</xml_diff>